<commit_message>
Approved email text word for word; only fill-in spots personalised
- TEMPLATE_A/B and follow-ups restored to the approved wording (verified identical to the brief);
  signature on three lines per the layout rule
- fill_ins(): [Name], [Brand], [country] (confirmed only, else country-free version), [category],
  [product], opening line; brands with a missing fill-in are held back and listed
- per-brand [category] set for batch 2026-09-28; daily table shows every fill-in value
- batch 2026-09-28 rebuilt, approvals reset pending the user's OK on the new table
- first-email tests re-sent to info@joinmatchly.com (BPerfect A, Makear B)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015V3tpdvHrRGbX5pxPwM4Y2
</commit_message>
<xml_diff>
--- a/later_expandnow.xlsx
+++ b/later_expandnow.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>no specific opener found on site; bestseller (magnesium capsules) has no clear video angle; needs a better featured product</t>
+          <t>missing fill-in: opener; no specific opener found on site; bestseller (magnesium capsules) has no clear video angle; needs a better featured product</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>home country not confirmed on the brand's legal/imprint/terms page; no specific opener found on site; no featured product; no specific featured product found on site</t>
+          <t>home country not confirmed on the brand's legal/imprint/terms page; missing fill-in: product, opener; no specific opener found on site; no featured product; no specific featured product found on site</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>home country not confirmed on the brand's legal/imprint/terms page; no specific opener found on site; no featured product; no specific featured product found on site</t>
+          <t>home country not confirmed on the brand's legal/imprint/terms page; missing fill-in: product, opener; no specific opener found on site; no featured product; no specific featured product found on site</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">

</xml_diff>